<commit_message>
docs(handoff): 온톨로지 전달 ZIP·XLSX 를 현재 SoT 로 동기화 + usage_count 명칭 통일 (B-갭5)
- XLSX(CCOP_Ontology_V4.8_node_edge_attrs.xlsx) 46셀 갱신:
  · 노드카탈로그 vt_case 표준 식별자 flnm(사건번호) → incdnt_no(경찰청 공식 사건번호)
  · 노드 속성 사전 flnm = 보조 속성(식별자 아님), vt_petition.linked_case_id → vt_case.incdnt_no
  · 엣지카탈로그 used_ip·contacted·located_at 주요 속성을 SoT·적재기 집계 속성과 일치
  · 엣지 속성 사전 first_dt/last_dt·evt_count·access_type·call_count 등 추가, 변경이력 R18·R19
- ontology_v4.8.zip 재생성(9/14 판 → 현재 code/·spec/): 내부 Python vt_case canonical_field
  flnm → incdnt_no 로 해제본과 일치
- used_ip 집계 건수 access_count → usage_count: 이미 전달된 XLSX 엣지 속성 사전의 명칭 재사용
  (SoT·적재기·규격서·테스트·전달본 SoT 재생성)

미결: flnm 자체의 정의(표준 DDL TB_INCDNT_M.FLNM='성명' vs 규격 '내부 사건파일명') — 결정 후 반영

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/handoff/ontology_v4.8/spec/CCOP_Ontology_V4.8_node_edge_attrs.xlsx
+++ b/handoff/ontology_v4.8/spec/CCOP_Ontology_V4.8_node_edge_attrs.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="변경이력(V4.3→V4.8)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="엣지카탈로그(72종)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="노드카탈로그(25종)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="노드 속성 사전" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="엣지 속성 사전" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="값 도메인 사전" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="탐색·적재 규칙" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="파생속성 등록부" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공통 메타·안내" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="변경이력(V4.3→V4.8)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="엣지카탈로그(72종)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="노드카탈로그(25종)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="노드 속성 사전" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="엣지 속성 사전" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="값 도메인 사전" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="탐색·적재 규칙" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="파생속성 등록부" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="공통 메타·안내" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="53" min="1" max="1"/>
@@ -2210,150 +2210,224 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="53" t="inlineStr">
         <is>
           <t>R14</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="53" t="inlineStr">
         <is>
           <t>V4.8</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="53" t="inlineStr">
         <is>
           <t>도메인 확장</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="53" t="inlineStr">
         <is>
           <t>contacted</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="53" t="inlineStr">
         <is>
           <t>Phone→Phone</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="53" t="inlineStr">
         <is>
           <t>Phone|DigitalID→Phone|DigitalID (channel 속성 신설)</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G43" s="53" t="inlineStr">
         <is>
           <t>EP1~8 전수감사: 카톡 대화상대(계정간) 4,107건 실적재 — 집계 관계라 msg reification 불가 (docs/EP1_EP8_V47_AUDIT_20260902.md)</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="53" t="inlineStr">
         <is>
           <t>R15</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="53" t="inlineStr">
         <is>
           <t>V4.8</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="53" t="inlineStr">
         <is>
           <t>도메인 확장</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="53" t="inlineStr">
         <is>
           <t>registered_to</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="53" t="inlineStr">
         <is>
           <t>Phone→Person</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="53" t="inlineStr">
         <is>
           <t>Phone|DigitalID→Person</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" s="53" t="inlineStr">
         <is>
           <t>네이버 실명확인 가입자 1,914건 — uses_id(사용자)와 명의자 구분이 대포계정 표현 핵심</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="53" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="53" t="inlineStr">
         <is>
           <t>V4.8</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="53" t="inlineStr">
         <is>
           <t>도메인 확장</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="53" t="inlineStr">
         <is>
           <t>used_ip</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="53" t="inlineStr">
         <is>
           <t>Person|Phone|DigitalID|Device→NetworkTrace</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="53" t="inlineStr">
         <is>
           <t>+BankAccount (뱅킹 접속 IP; 시각 레코드는 R8 reification 우선)</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="53" t="inlineStr">
         <is>
           <t>EP3 012 ipmac 5건 + EP9/10 뱅킹 IP 27.193.61.154</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="53" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="53" t="inlineStr">
         <is>
           <t>V4.8</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="53" t="inlineStr">
         <is>
           <t>개명</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="53" t="inlineStr">
         <is>
           <t>sameAs</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="53" t="inlineStr">
         <is>
           <t>sameAs (camelCase)</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="53" t="inlineStr">
         <is>
           <t>same_as (snake_case 전면 통일)</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" s="53" t="inlineStr">
         <is>
           <t>AgensGraph 미인용 식별자 소문자화로 DB 실현명 sameas — UI 스타일 셀렉터 미매칭 문제 해결, DB 4건 마이그레이션</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="53" t="inlineStr">
+        <is>
+          <t>R18</t>
+        </is>
+      </c>
+      <c r="B47" s="53" t="inlineStr">
+        <is>
+          <t>V4.8</t>
+        </is>
+      </c>
+      <c r="C47" s="53" t="inlineStr">
+        <is>
+          <t>식별자 변경</t>
+        </is>
+      </c>
+      <c r="D47" s="53" t="inlineStr">
+        <is>
+          <t>vt_case</t>
+        </is>
+      </c>
+      <c r="E47" s="53" t="inlineStr">
+        <is>
+          <t>flnm(사건번호)</t>
+        </is>
+      </c>
+      <c r="F47" s="53" t="inlineStr">
+        <is>
+          <t>incdnt_no(경찰청 공식 사건번호), flnm 은 보조 속성</t>
+        </is>
+      </c>
+      <c r="G47" s="53" t="inlineStr">
+        <is>
+          <t>사건번호·파일명 개념 분리 (2026-09-18) — 적재기·검증기·통합그래프 반영</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="53" t="inlineStr">
+        <is>
+          <t>R19</t>
+        </is>
+      </c>
+      <c r="B48" s="53" t="inlineStr">
+        <is>
+          <t>V4.8</t>
+        </is>
+      </c>
+      <c r="C48" s="53" t="inlineStr">
+        <is>
+          <t>집계 규칙</t>
+        </is>
+      </c>
+      <c r="D48" s="53" t="inlineStr">
+        <is>
+          <t>used_ip · located_at</t>
+        </is>
+      </c>
+      <c r="E48" s="53" t="inlineStr">
+        <is>
+          <t>행마다 덮어쓰기(마지막 행 시각만)·evt_ymdhm 미저장</t>
+        </is>
+      </c>
+      <c r="F48" s="53" t="inlineStr">
+        <is>
+          <t>쌍당 1엣지 + valid_from/valid_to·usage_count / first_dt/last_dt/evt_count</t>
+        </is>
+      </c>
+      <c r="G48" s="53" t="inlineStr">
+        <is>
+          <t>협력기관 질의(2026-09-28): 위치 1,207건→380엣지로 합쳐지며 시각 소실</t>
         </is>
       </c>
     </row>
@@ -2960,7 +3034,7 @@
       </c>
       <c r="E17" s="85" t="inlineStr">
         <is>
-          <t>first_seen, last_seen, usage_count, subject_type</t>
+          <t>valid_from, valid_to, usage_count, access_type, source_id</t>
         </is>
       </c>
       <c r="F17" s="85" t="inlineStr">
@@ -2970,7 +3044,7 @@
       </c>
       <c r="G17" s="85" t="inlineStr">
         <is>
-          <t>V4.4 domain 확장 (G3) · V4.5 vt_dev 추가 + 무방향 탐색 (G10) [V4.8 domain+BankAccount, R8 reification 우선 노트]</t>
+          <t>V4.4 domain 확장 (G3) · V4.5 vt_dev 추가 + 무방향 탐색 (G10) [V4.8 domain+BankAccount, R8 reification 우선 노트] · V4.8 (주체,IP)쌍 집계: valid_from=최초·valid_to=마지막 관측·usage_count</t>
         </is>
       </c>
     </row>
@@ -3949,7 +4023,7 @@
       </c>
       <c r="E46" s="85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>channel, first_dt, last_dt, call_count, msg_count, total_dur_sec, source_id</t>
         </is>
       </c>
       <c r="F46" s="86" t="inlineStr">
@@ -3959,7 +4033,7 @@
       </c>
       <c r="G46" s="85" t="inlineStr">
         <is>
-          <t>[V4.8 domain/range+DigitalID, channel 속성]</t>
+          <t>[V4.8 domain/range+DigitalID, channel 속성] · (쌍,channel) 집계 속성 명시</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4579,7 @@
       </c>
       <c r="E62" s="53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>first_dt, last_dt, evt_count, source_id</t>
         </is>
       </c>
       <c r="F62" s="92" t="inlineStr">
@@ -4515,7 +4589,7 @@
       </c>
       <c r="G62" s="92" t="inlineStr">
         <is>
-          <t>정합화 등재</t>
+          <t>정합화 등재 · V4.8 (주체,위치)쌍 집계 — 시각 있는 행만 first_dt/last_dt/evt_count</t>
         </is>
       </c>
     </row>
@@ -5065,7 +5139,7 @@
       </c>
       <c r="D3" s="85" t="inlineStr">
         <is>
-          <t>flnm(사건번호)</t>
+          <t>incdnt_no(경찰청 공식 사건번호)</t>
         </is>
       </c>
       <c r="E3" s="85" t="inlineStr">
@@ -6106,7 +6180,7 @@
       </c>
       <c r="D12" s="86" t="inlineStr">
         <is>
-          <t>사건번호(내부, 예: 2026-CYBER-00123)</t>
+          <t>보조 속성 — 식별자 아님(V4.8). 종전 내부 사건번호 용도였으나 사건 식별은 incdnt_no 로 이관</t>
         </is>
       </c>
       <c r="E12" s="92" t="inlineStr">
@@ -6133,7 +6207,7 @@
       </c>
       <c r="D13" s="86" t="inlineStr">
         <is>
-          <t>경찰청 공식 사건번호</t>
+          <t>경찰청 공식 사건번호 — vt_case 정경 식별자(V4.8)</t>
         </is>
       </c>
       <c r="E13" s="92" t="inlineStr">
@@ -6781,7 +6855,7 @@
       </c>
       <c r="D37" s="86" t="inlineStr">
         <is>
-          <t>연결된 vt_case.flnm</t>
+          <t>연결된 vt_case.incdnt_no</t>
         </is>
       </c>
       <c r="E37" s="92" t="inlineStr">
@@ -13013,7 +13087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="16.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="53" min="1" max="1"/>
@@ -13552,7 +13626,7 @@
       </c>
       <c r="D20" s="85" t="inlineStr">
         <is>
-          <t>used_in_device, used_ip</t>
+          <t>used_in_device</t>
         </is>
       </c>
       <c r="E20" s="92" t="inlineStr">
@@ -13736,7 +13810,7 @@
       </c>
       <c r="C27" s="85" t="inlineStr">
         <is>
-          <t>IP 사용 횟수</t>
+          <t>IP 사용(접속) 행 수 — (주체,IP)쌍 집계 시 합계 (V4.8)</t>
         </is>
       </c>
       <c r="D27" s="85" t="inlineStr">
@@ -14561,29 +14635,137 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="53" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
+      <c r="B58" s="53" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C58" s="53" t="inlineStr">
         <is>
           <t>연락 수단 구분 — 'call'|'kakao'|'sms' (V4.8)</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="53" t="inlineStr">
         <is>
           <t>contacted</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="53" t="inlineStr">
         <is>
           <t>enum</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="53" t="inlineStr">
+        <is>
+          <t>first_dt / last_dt</t>
+        </is>
+      </c>
+      <c r="B59" s="53" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C59" s="53" t="inlineStr">
+        <is>
+          <t>쌍 집계 엣지의 최초/최종 관측 시각 (V4.8)</t>
+        </is>
+      </c>
+      <c r="D59" s="53" t="inlineStr">
+        <is>
+          <t>contacted, located_at</t>
+        </is>
+      </c>
+      <c r="E59" s="53" t="inlineStr">
+        <is>
+          <t>날짜시간</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="53" t="inlineStr">
+        <is>
+          <t>evt_count</t>
+        </is>
+      </c>
+      <c r="B60" s="53" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C60" s="53" t="inlineStr">
+        <is>
+          <t>시각 있는 위치 관측 행 수 (V4.8)</t>
+        </is>
+      </c>
+      <c r="D60" s="53" t="inlineStr">
+        <is>
+          <t>located_at</t>
+        </is>
+      </c>
+      <c r="E60" s="53" t="inlineStr">
+        <is>
+          <t>수치</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="53" t="inlineStr">
+        <is>
+          <t>access_type</t>
+        </is>
+      </c>
+      <c r="B61" s="53" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C61" s="53" t="inlineStr">
+        <is>
+          <t>접속 유형 web|comm|banking — 여러 값이면 '|' 결합 (V4.8)</t>
+        </is>
+      </c>
+      <c r="D61" s="53" t="inlineStr">
+        <is>
+          <t>used_ip</t>
+        </is>
+      </c>
+      <c r="E61" s="53" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="53" t="inlineStr">
+        <is>
+          <t>call_count / msg_count / total_dur_sec</t>
+        </is>
+      </c>
+      <c r="B62" s="53" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C62" s="53" t="inlineStr">
+        <is>
+          <t>통화 건수 / 메시지 건수 / 통화 총 초 (V4.8 집계)</t>
+        </is>
+      </c>
+      <c r="D62" s="53" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="E62" s="53" t="inlineStr">
+        <is>
+          <t>수치</t>
         </is>
       </c>
     </row>

</xml_diff>